<commit_message>
Schedule at 5 route-day slots per PL-week; pack revisits into full loop days
Per Joe: plan a full 5-day field week and stop showing scattered 1-2 stop
revisit entries. Cycle 2 (W1-W9, Aug 3 -> Sep 28) now plans 1,197 stops in
141 full-day entries: 57 first-pass days plus 83 producer-loop days -
same-week cadence revisits packed into single <=10-stop drives labeled
like R03+R07. Sean stays at 2 slots (40-account book saturates). Backlog
collapses from 234 stops to one day (Kristen R18; its producers sweep in
W2). Flex slots are shown in each workbook's Weekly Plan tab. Flagged in
the plan and SOP r2: this supersedes the 3-4-day ortho guard, and
Kristen's book fills all 5 slots every week - needs Kristen/Gautam
sign-off. Schedule rows now carry base_day/base_stop so twin locations
map exactly in the app.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ei2NMkxuP1dquQsjedq4wC
</commit_message>
<xml_diff>
--- a/pm/route-days-v2/Spine-Route-Days-Jasmine.xlsx
+++ b/pm/route-days-v2/Spine-Route-Days-Jasmine.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +45,11 @@
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="5">
@@ -87,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -106,6 +111,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1045,7 +1056,7 @@
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
@@ -1225,7 +1236,7 @@
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="K17" s="5" t="inlineStr">
@@ -1270,7 +1281,7 @@
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -1315,7 +1326,7 @@
       </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
@@ -1360,7 +1371,7 @@
       </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -1405,7 +1416,7 @@
       </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
@@ -1450,7 +1461,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -1495,7 +1506,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K23" s="5" t="inlineStr">
@@ -1540,7 +1551,7 @@
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -1585,7 +1596,7 @@
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr">
@@ -1630,7 +1641,7 @@
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -1675,7 +1686,7 @@
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
@@ -1720,7 +1731,7 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -1765,7 +1776,7 @@
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
@@ -1810,7 +1821,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -1855,7 +1866,7 @@
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="K31" s="5" t="inlineStr">
@@ -1900,7 +1911,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -1945,7 +1956,7 @@
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>Backlog (Oct+ / after 90-day read)</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -20975,21 +20986,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="72" customWidth="1" min="6" max="6"/>
+    <col width="68" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cycle 2 plan. First pass = the full day. Cadence revisit / Producer sweep = the producing accounts only (2–4 quick stops). Pick the weekday at the Monday huddle.</t>
+          <t>5 route-day slots per week. First pass = the full day. Cadence revisit = the producers due on rhythm, packed into one full loop day (a label like R03+R07 = one drive covering both days’ producers). Open slots are flex. Pick weekdays at the Monday huddle.</t>
         </is>
       </c>
     </row>
@@ -21006,7 +21017,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Route Day</t>
+          <t>Route Day(s)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -21036,7 +21047,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>J-R02</t>
         </is>
@@ -21066,7 +21077,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>J-R03</t>
         </is>
@@ -21096,7 +21107,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>J-R06</t>
         </is>
@@ -21126,7 +21137,7 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>J-R08</t>
         </is>
@@ -21148,30 +21159,30 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>J-R04</t>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>J-R11</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>OAK STREET HEALTH CHERRY HILL · APOLLO HEALTH SERVICES, PC · Plymouth physical therapy services</t>
+          <t>FARMBROOK INTERVENTIONAL PAIN AND EMG · Glazer Spine Center- use · Leonard Sahn MD · Pain Clinic of Michigan · IMMEDIATE CARE MEDICAL CENTER, PC · Premier Medicine Medical Center - Livonia · Botsford General Hospital · Corewell Health Urgent Care · MICHIGAN ORTHOPEDIC SPECIALISTS - Farmington Hills · SPECIALISTS IN SPINE SURGERY - Farmington Hills</t>
         </is>
       </c>
     </row>
@@ -21186,9 +21197,9 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>J-R05</t>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>J-R04+R05+R07</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -21197,11 +21208,11 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Eastpointe Family Physicians · QuickDoc Urgent Care</t>
+          <t>Eastpointe Family Physicians · QuickDoc Urgent Care · OAK STREET HEALTH CHERRY HILL · APOLLO HEALTH SERVICES, PC · Plymouth physical therapy services · NORLIVO INTERNAL MEDICINE</t>
         </is>
       </c>
     </row>
@@ -21216,22 +21227,22 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>J-R07</t>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>J-R13</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>NORLIVO INTERNAL MEDICINE</t>
+          <t>UofM Canton Health Center General Medicine · UofM Pain Management - Canton · All-Pro Physical Therapy · Advanced Primary Care · Care Medical Clinic of Canton · A1 Family Medicine · CoreWell Health Family Medicine · Michigan family wellness · Sarju Shah Family Medicine and Geriatrics · BEAUMONT CHERRY HILL INTERNAL MEDICAL ASSOCIATES CANTON</t>
         </is>
       </c>
     </row>
@@ -21246,9 +21257,9 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>J-R11</t>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>J-R14</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -21257,11 +21268,11 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>FARMBROOK INTERVENTIONAL PAIN AND EMG · Glazer Spine Center- use · Leonard Sahn MD · Pain Clinic of Michigan · IMMEDIATE CARE MEDICAL CENTER, PC · Premier Medicine Medical Center - Livonia · Botsford General Hospital · Corewell Health Urgent Care · MICHIGAN ORTHOPEDIC SPECIALISTS - Farmington Hills · SPECIALISTS IN SPINE SURGERY - Farmington Hills</t>
+          <t>MDVIP-Novi · Rivi Medical Associates · Park Internal Medicine · Park Family Practice - Novi · Karma Internists · Providence Internal Medicine, Diabetes/Endocrinology · IEP Urgent Care- Novi · Corewell Health Family Care of Novi · Corewell Urgent Care - Novi</t>
         </is>
       </c>
     </row>
@@ -21276,9 +21287,9 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>J-R13</t>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>J-R15</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -21287,11 +21298,11 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>UofM Canton Health Center General Medicine · UofM Pain Management - Canton · All-Pro Physical Therapy · Advanced Primary Care · Care Medical Clinic of Canton · A1 Family Medicine · CoreWell Health Family Medicine · Michigan family wellness · Sarju Shah Family Medicine and Geriatrics · BEAUMONT CHERRY HILL INTERNAL MEDICAL ASSOCIATES CANTON</t>
+          <t>ACADEMIC INTERNAL MEDICINE SPECIALISTS · SOUTHFIELD URGENT CARE · Get Well Urgent Care Southfield · Concentra Urgent Care - Southfield · Doctors Urgent Care - Southfield · EXPRESS MED URGENT CARE · DEDICATED SENIOR MEDICAL CENTER - Southfield · Roberts Orthopedic Services · Michigan Orthopedic Surgeons- Southfield</t>
         </is>
       </c>
     </row>
@@ -21306,9 +21317,9 @@
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>J-R14</t>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>J-R16</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -21317,11 +21328,11 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>MDVIP-Novi · Rivi Medical Associates · Park Internal Medicine · Park Family Practice - Novi · Karma Internists · Providence Internal Medicine, Diabetes/Endocrinology · IEP Urgent Care- Novi · Corewell Health Family Care of Novi · Corewell Urgent Care - Novi</t>
+          <t>Intensive Pulmonary &amp; Internal Medicine · Trinity Health IHA Medical Group, Hospital Medicine · Trinity Health - Emergency Medicine · Western Wayne Physicians - Livonia · Lakes Urgent Care - Livonia · Doctors urgent care · Team Rehabilitation physical therapy · PROVIDENCE PARK LIVONIA FAMILY MEDICINE · Trinity IHA Academic Family Medicine - Livonia · Trinity Health IHA Academic Internal Medicine</t>
         </is>
       </c>
     </row>
@@ -21336,9 +21347,9 @@
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>J-R01</t>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>J-R01+R04+R05+R07+R09+R12</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -21347,11 +21358,11 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Corwell health orthopedics Canton · CANTON FAMILY HEALTH LLC · Comprehensive Healthcare Associates and Prevention Medicine</t>
+          <t>Michigan Primary Care - Eastpointe · Dedicated Senior Medical Center - Eastpointe · Corwell health orthopedics Canton · CANTON FAMILY HEALTH LLC · Comprehensive Healthcare Associates and Prevention Medicine · Wayne Primary Care and Walk In · Freedom Medical Clinic (Trinity) · DEARBORN FAMILY CLINIC, PC · PelHam Primary Care · Grand River Medical Associates</t>
         </is>
       </c>
     </row>
@@ -21366,9 +21377,9 @@
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>J-R04</t>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>J-R10</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -21381,7 +21392,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Wayne Primary Care and Walk In</t>
+          <t>Frank Lanzilote DO-Family Practice</t>
         </is>
       </c>
     </row>
@@ -21396,22 +21407,22 @@
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>J-R05</t>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>J-R17</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Michigan Primary Care - Eastpointe · Dedicated Senior Medical Center - Eastpointe</t>
+          <t>Gretchen’s place · VAN BUREN URGENT CARE · MI Express Care · IHA ORTHOPAEDIC SURGERY ASSOCIATES - CANTON · Trinity URGENT CARE CANTON · Trinity Health IHA Medical Group Primary Care - Canton · IHA, Primary Care - Cherry Hill Village · Partners in Internal Medicine · PONDURI, KAVITHA, MEDICAL GROUP · BEAUMONT URGENT CARE BY WELLSTREET</t>
         </is>
       </c>
     </row>
@@ -21426,22 +21437,22 @@
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>J-R07</t>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>J-R18</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Freedom Medical Clinic (Trinity)</t>
+          <t>TRINITY HEALTH URGENT CARE- Livonia · Trinity Health IHA Medical Group, Primary Care - Southeast Livonia · Henry Ford urgent care Livonia · Lawrence Lipnik MD, · CARSON, DARCELLE M, MEDICAL GROUP · Wellness Wave Chiropractic · True Health Chiropractic · Chiro-Care of Livonia · CENTER FOR INTERNAL MEDICINE CONTINUITY CLINIC</t>
         </is>
       </c>
     </row>
@@ -21456,39 +21467,39 @@
           <t>2026-08-17</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>J-R09</t>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>J-R19</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>DEARBORN FAMILY CLINIC, PC · PelHam Primary Care</t>
+          <t>Trinity Health IHA Primary Care - EMU · UNIVERSITY OF MICHIGAN YPSILANTI HEALTH CENTER · Trinity Health Neighborhood Primary Care · CORNER HEALTH CENTER (Medicaid) · ATI Ypsilanti Huron Rd · SOUTH HURON URGENT CARE (CAT 3) · Medical Associates PC · Vladimir Klemptner MD, · BEAUMONT FAMILY MEDICINE BELLEVILLE · WELLHEALTH MEDICAL ASSOCIATES - Belleville</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>J-R10</t>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>J-R01+R02+R03+R06+R08+R10</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -21497,28 +21508,28 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Frank Lanzilote DO-Family Practice</t>
+          <t>Park Medical Center (Medicaid) · Core Institute/Henry Ford Motor City Orthopedics &amp; PT- Southfield · BN Nandish MD · Park Medical Centers - Canton · Corewell Health Wayne Hospital Family Medicine -  Canton · Synergy Medical Primary Care · Livonia Family Medical Center · Dedicated senior Medical Center Detroit North · The family Doc · DMC SPORTS MEDICINE NOVI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>J-R12</t>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>J-R11</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -21531,24 +21542,24 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Grand River Medical Associates</t>
+          <t>Premier Medicine Medical Center - Livonia</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>J-R15</t>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>J-R20</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -21561,24 +21572,24 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>ACADEMIC INTERNAL MEDICINE SPECIALISTS · SOUTHFIELD URGENT CARE · Get Well Urgent Care Southfield · Concentra Urgent Care - Southfield · Doctors Urgent Care - Southfield · EXPRESS MED URGENT CARE · DEDICATED SENIOR MEDICAL CENTER - Southfield · Roberts Orthopedic Services · Michigan Orthopedic Surgeons- Southfield</t>
+          <t>CEDAR MEDICAL ASSOCIATES · SUNSTRUM MEDICAL ASSOCIATES, PC · Fayda Zakaria MD Family Medicine · MDWell · TENNY INTERNAL MEDICINE, PLLC · BEAUMONT URGENT CARE BY WELLSTREET · HEIGHTS FAMILY MEDICINE · FORD TEL MEDICAL CENTER · MICHIGAN INTERVENTIONAL PAIN CENTER (this is an ASC)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W4</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>J-R16</t>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>J-R21</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -21591,7 +21602,7 @@
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Intensive Pulmonary &amp; Internal Medicine · Trinity Health IHA Medical Group, Hospital Medicine · Trinity Health - Emergency Medicine · Western Wayne Physicians - Livonia · Lakes Urgent Care - Livonia · Doctors urgent care · Team Rehabilitation physical therapy · PROVIDENCE PARK LIVONIA FAMILY MEDICINE · Trinity IHA Academic Family Medicine - Livonia · Trinity Health IHA Academic Internal Medicine</t>
+          <t>RIVER OAKS PRIMARY CARE · COREWELL HEALTH  INTERNAL MEDICINE DEARBORN · BRYANT PRIMARY CARE Updated · Associated physicians of Dearborn · Dearborn Family Doctors · Raad Al-Saraf MD PC · WARRENFIELD MEDICAL CENTER (Medicaid) · EAST DEARBORN MEDICAL CLINIC, PC (Medicaid) · Dearborn Health Clinic · Bingham Medical Center</t>
         </is>
       </c>
     </row>
@@ -21606,39 +21617,39 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>J-R01</t>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>J-R22</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>BN Nandish MD</t>
+          <t>ORTHOPEDIC SURGERY SPECIALISTS, PLLC · Gem Health and Wellness · Oakland Rehabilitation Associates · Office of Robert Brateman · Family Care Physicians PC · Primecare of Novi · PRIMECARE URGENT CARE, PLLC · Everside Health · Southeast Michigan Rehab &amp; Pain</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>J-R02</t>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>J-R02+R04+R06+R07+R13+R14+R16</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -21647,28 +21658,28 @@
         </is>
       </c>
       <c r="E23" s="3" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>DMC SPORTS MEDICINE NOVI</t>
+          <t>BEAUMONT FAMILY MEDICINE GARDEN CITY · MEDICAL GROUP PRACTICE, PC (Olympia health) · NORLIVO INTERNAL MEDICINE · A1 Family Medicine · Lakes Urgent Care - Livonia · Village Medical - Novi · WEST OAKLAND INTERNISTS · Karma Internists</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>J-R03</t>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>J-R03+R04+R05+R08+R15</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -21677,123 +21688,123 @@
         </is>
       </c>
       <c r="E24" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Park Medical Centers - Canton · Corewell Health Wayne Hospital Family Medicine -  Canton</t>
+          <t>Eastpointe Family Physicians · QuickDoc Urgent Care · Tri County Neurology · Dedicated Senior Medical Center - Warren · Roberts Orthopedic Services · Corewell Health Wayne Hospital Internal Medicine - Canton · CANTON FOOT &amp; Ankle SPECIALISTS · OAK STREET HEALTH CHERRY HILL · APOLLO HEALTH SERVICES, PC · Plymouth physical therapy services</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>J-R06</t>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>J-R23</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E25" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>Synergy Medical Primary Care · Livonia Family Medical Center</t>
+          <t>Northville-Novi Family Medicine · MICHIGAN INSTITUTE OF MEDICINE · Corwell internal medicine and primary care · Michigan Urgent Care - Livonia · Henry Ford employer solutions · Trinity IHA Orthopedics - Schoolcraft · IHA urgent care Livonia · Corewell Health Farmington hills Hospital family medicine · ORTHOPEDIC INSTITUTE OF MICHIGAN · PRIZM PAIN SPECIALISTS, PLLC</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>J-R08</t>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>J-R24</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E26" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Park Medical Center (Medicaid) · Core Institute/Henry Ford Motor City Orthopedics &amp; PT- Southfield</t>
+          <t>Elite Prime Care · PLYMOUTH CANTON FAMILY HEALTH · Michigan Orthopedic Specialists · Plymouth urgent care walk-in clinic · Gingell Chiropractic · THE PILOT DOCTORS · Office of Jeff The DO · Office of Robert Vartabedian MD · IHA Plymouth Primary Care · Ethos Physical Therapy</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>J-R10</t>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>J-R25</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E27" s="3" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>Dedicated senior Medical Center Detroit North · The family Doc</t>
+          <t>City Medical - Southgate · PEDIATRIC AND ADOLESCENT CENTER · ALLENWOOD FAMILY HEALTH CARE, PC · DOWNRIVER INTERNISTS, PC · PARK PLACE FAMILY PRACTICE AND INTERNAL MEDICINE · BEAUMONT ATHENS CLINIC TAYLOR · BADHWAR ASSOCIATES, MD, PC · King Medical Center · HENRY FORD HEALTH</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>J-R17</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>J-R01+R09+R12+R13+R15</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>First pass</t>
+          <t>Cadence revisit</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
@@ -21801,144 +21812,144 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Gretchen’s place · VAN BUREN URGENT CARE · MI Express Care · IHA ORTHOPAEDIC SURGERY ASSOCIATES - CANTON · Trinity URGENT CARE CANTON · Trinity Health IHA Medical Group Primary Care - Canton · IHA, Primary Care - Cherry Hill Village · Partners in Internal Medicine · PONDURI, KAVITHA, MEDICAL GROUP · BEAUMONT URGENT CARE BY WELLSTREET</t>
+          <t>ACADEMIC INTERNAL MEDICINE SPECIALISTS · Corwell health orthopedics Canton · CANTON FAMILY HEALTH LLC · Comprehensive Healthcare Associates and Prevention Medicine · DEARBORN FAMILY CLINIC, PC · PelHam Primary Care · Grand River Medical Associates · UofM Canton Health Center General Medicine · Care Medical Clinic of Canton · CoreWell Health Family Medicine</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>J-R18</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>J-R10+R14+R16+R17+R18+R19</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>First pass</t>
+          <t>Cadence revisit</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>TRINITY HEALTH URGENT CARE- Livonia · Trinity Health IHA Medical Group, Primary Care - Southeast Livonia · Henry Ford urgent care Livonia · Lawrence Lipnik MD, · CARSON, DARCELLE M, MEDICAL GROUP · Wellness Wave Chiropractic · True Health Chiropractic · Chiro-Care of Livonia · CENTER FOR INTERNAL MEDICINE CONTINUITY CLINIC</t>
+          <t>Western Wayne Physicians - Livonia · PROVIDENCE PARK LIVONIA FAMILY MEDICINE · Trinity Health IHA Medical Group Primary Care - Canton · Trinity Health IHA Medical Group, Primary Care - Southeast Livonia · BEAUMONT FAMILY MEDICINE BELLEVILLE · Frank Lanzilote DO-Family Practice · Corewell Health Family Care of Novi</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>J-R02</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>J-R26</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Village Medical - Novi · WEST OAKLAND INTERNISTS</t>
+          <t>Levan Internists · AMINI HEALTHCARE, PLLC · MD VIP - Trenton · DOWNRIVER INTERNAL MEDICINE, PC · FAMILY HEALTH, PC · METRO SHORES INTERNAL MEDICINE, PLLC · Ben Go MD PC · MIND-Riverview</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>J-R03</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>J-R27</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E31" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>Corewell Health Wayne Hospital Internal Medicine - Canton · CANTON FOOT &amp; Ankle SPECIALISTS</t>
+          <t>MI Express Urgent Care · Trinity IHA Orthopedics - West Arbor · Trinity IHA Primary Care - West Arbor · Trinity Health Urgent Care - West Arbor suite 230 · Sickels MD, Malcolm · Internal Medicine Clinic - Taubman Center · NASSER SUKHON, MD, PC · Partners in internal medicine · Integrative Family Medicine Clinic - Domino's Farms (U of M) · Adult Medicine &amp; Pediatrics at East Ann Arbor Health and Geriatrics Center</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>J-R04</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>J-R28</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E32" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>OAK STREET HEALTH CHERRY HILL · BEAUMONT FAMILY MEDICINE GARDEN CITY · APOLLO HEALTH SERVICES, PC · Plymouth physical therapy services</t>
+          <t>Trinity health urgent care – EMU · Hewitt Road Medical Center · IHA ARBOR PARK PRIMARY CARE · IHA Family Medicine · Trinity IHA Pediatrics - Arbor Park · Trinity health physical therapy · Trinity Health Orthopedic group-Ypsilanti · ACADEMIC INTERNAL MEDICINE · Trinity Health IHA Medical Group, Primary Care - Ann Arbor</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>J-R05</t>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>J-R02+R11+R17+R18+R20+R21</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -21947,28 +21958,28 @@
         </is>
       </c>
       <c r="E33" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F33" s="4" t="inlineStr">
         <is>
-          <t>Eastpointe Family Physicians · QuickDoc Urgent Care</t>
+          <t>IHA, Primary Care - Cherry Hill Village · CENTER FOR INTERNAL MEDICINE CONTINUITY CLINIC · TENNY INTERNAL MEDICINE, PLLC · COREWELL HEALTH  INTERNAL MEDICINE DEARBORN · DMC SPORTS MEDICINE NOVI · ASCENSION MEDICAL GROUP WEST BLOOMFIELD FAMILY PRACTICE · Novi Medicine · Premier Medicine Medical Center - Livonia</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>J-R06</t>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>J-R03+R04+R05+R06+R07+R08</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -21977,118 +21988,118 @@
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL GROUP PRACTICE, PC (Olympia health)</t>
+          <t>Michigan Primary Care - Eastpointe · Dedicated Senior Medical Center - Eastpointe · Park Medical Center (Medicaid) · Core Institute/Henry Ford Motor City Orthopedics &amp; PT- Southfield · Park Medical Centers - Canton · Corewell Health Wayne Hospital Family Medicine -  Canton · Wayne Primary Care and Walk In · Synergy Medical Primary Care · Livonia Family Medical Center · Freedom Medical Clinic (Trinity)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>J-R07</t>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>J-R29</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>NORLIVO INTERNAL MEDICINE</t>
+          <t>Evolve Medical - Dearborn · Premier Medicine Primary and Urgent Care · GREENFIELD MEDICAL CENTER OF DEARBORN, PC · Oakman, Medical Center · PRIME CARE MEDICAL CLINIC · Schaefer Medical · Corwell health internal medicine, Dearborn · EASTBORN MEDICAL GROUP · ALI M NASSER, MD, PC · PULSE PRIMARY/SENIOR CARE</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>J-R08</t>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>J-R30</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Tri County Neurology · Dedicated Senior Medical Center - Warren</t>
+          <t>TERRY D HOWELL, MD, PC · Bio Energy Medical Center · MDVIP Ann Arbor · Packard Health - Ann Arbor · Michigan urgent care · Integrative Healthcare Providers · Briarwood Family Medicine · STEINER HEALTH · Dr. Susannah Parke · Krasnick Regenerative Medicine</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W7</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>J-R11</t>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>J-R31</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Cadence revisit</t>
+          <t>First pass</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Premier Medicine Medical Center - Livonia</t>
+          <t>BEAUMONT FAMILY MEDICINE CLINIC TAYLOR · Taylor walk-in clinic · TAYLOR INTERNAL MEDICINE ASSOCIATES, PC · PROGRESSIVE HEALTH CARE, PC · AMC Primary Care · AMC Primary Care · DOWN RIVER MEDICAL GROUP · BEAUMONT HEALTH INTERNAL MEDICINE WYANDOTTE · SHEBA MEDICAL CENTER · DEARBORN HEALTHCARE, PC</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>J-R13</t>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>J-R01+R04+R05+R07+R15</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -22097,28 +22108,28 @@
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>A1 Family Medicine</t>
+          <t>Eastpointe Family Physicians · QuickDoc Urgent Care · Roberts Orthopedic Services · SOUTHFIELD URGENT CARE · DEDICATED SENIOR MEDICAL CENTER - Southfield · BN Nandish MD · OAK STREET HEALTH CHERRY HILL · APOLLO HEALTH SERVICES, PC · Plymouth physical therapy services · NORLIVO INTERNAL MEDICINE</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W8</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>J-R14</t>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>J-R10+R13+R14+R16+R22</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -22127,58 +22138,56 @@
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Karma Internists</t>
+          <t>A1 Family Medicine · Lakes Urgent Care - Livonia · Dedicated senior Medical Center Detroit North · The family Doc · Karma Internists · Park Family Practice - Novi · Corewell Urgent Care - Novi · Office of Robert Brateman · Family Care Physicians PC · Primecare of Novi</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>W5</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>J-R19</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>First pass</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>Trinity Health IHA Primary Care - EMU · UNIVERSITY OF MICHIGAN YPSILANTI HEALTH CENTER · Trinity Health Neighborhood Primary Care · CORNER HEALTH CENTER (Medicaid) · ATI Ypsilanti Huron Rd · SOUTH HURON URGENT CARE (CAT 3) · Medical Associates PC · Vladimir Klemptner MD, · BEAUMONT FAMILY MEDICINE BELLEVILLE · WELLHEALTH MEDICAL ASSOCIATES - Belleville</t>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>Open slot ×3</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr"/>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>Flex: backlog pull-forward · huddle promotes · ortho field day</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>J-R01</t>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>J-R01+R03+R06+R08+R09</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -22187,28 +22196,28 @@
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="F41" s="4" t="inlineStr">
         <is>
-          <t>Corwell health orthopedics Canton · CANTON FAMILY HEALTH LLC · Comprehensive Healthcare Associates and Prevention Medicine</t>
+          <t>Tri County Neurology · Dedicated Senior Medical Center - Warren · Corwell health orthopedics Canton · CANTON FAMILY HEALTH LLC · Comprehensive Healthcare Associates and Prevention Medicine · Corewell Health Wayne Hospital Internal Medicine - Canton · CANTON FOOT &amp; Ankle SPECIALISTS · MEDICAL GROUP PRACTICE, PC (Olympia health) · DEARBORN FAMILY CLINIC, PC · PelHam Primary Care</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>J-R09</t>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>J-R02+R24+R25</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -22217,28 +22226,28 @@
         </is>
       </c>
       <c r="E42" s="3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>DEARBORN FAMILY CLINIC, PC · PelHam Primary Care</t>
+          <t>Office of Jeff The DO · Office of Robert Vartabedian MD · IHA Plymouth Primary Care · City Medical - Southgate · PEDIATRIC AND ADOLESCENT CENTER · BADHWAR ASSOCIATES, MD, PC · Village Medical - Novi · WEST OAKLAND INTERNISTS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W9</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>J-R10</t>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>J-R10+R12+R17+R18+R19+R23</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -22247,1211 +22256,39 @@
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F43" s="4" t="inlineStr">
         <is>
-          <t>Frank Lanzilote DO-Family Practice</t>
+          <t>Grand River Medical Associates · Trinity Health IHA Medical Group Primary Care - Canton · PONDURI, KAVITHA, MEDICAL GROUP · Trinity Health IHA Medical Group, Primary Care - Southeast Livonia · BEAUMONT FAMILY MEDICINE BELLEVILLE · Corwell internal medicine and primary care · Michigan Urgent Care - Livonia · Trinity IHA Orthopedics - Schoolcraft · Frank Lanzilote DO-Family Practice</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>J-R12</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Grand River Medical Associates</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>J-R13</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>UofM Canton Health Center General Medicine · Care Medical Clinic of Canton · CoreWell Health Family Medicine</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>J-R14</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Corewell Health Family Care of Novi</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>J-R15</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Roberts Orthopedic Services</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>J-R16</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Lakes Urgent Care - Livonia</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>J-R20</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>First pass</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>CEDAR MEDICAL ASSOCIATES · SUNSTRUM MEDICAL ASSOCIATES, PC · Fayda Zakaria MD Family Medicine · MDWell · TENNY INTERNAL MEDICINE, PLLC · BEAUMONT URGENT CARE BY WELLSTREET · HEIGHTS FAMILY MEDICINE · FORD TEL MEDICAL CENTER · MICHIGAN INTERVENTIONAL PAIN CENTER (this is an ASC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>J-R02</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>DMC SPORTS MEDICINE NOVI · ASCENSION MEDICAL GROUP WEST BLOOMFIELD FAMILY PRACTICE · Novi Medicine</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>J-R03</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Park Medical Centers - Canton · Corewell Health Wayne Hospital Family Medicine -  Canton</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>J-R04</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Wayne Primary Care and Walk In</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>J-R05</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Michigan Primary Care - Eastpointe · Dedicated Senior Medical Center - Eastpointe</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>J-R06</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>Synergy Medical Primary Care · Livonia Family Medical Center</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>J-R07</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Freedom Medical Clinic (Trinity)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>J-R08</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>Park Medical Center (Medicaid) · Core Institute/Henry Ford Motor City Orthopedics &amp; PT- Southfield</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>J-R15</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F57" s="4" t="inlineStr">
-        <is>
-          <t>ACADEMIC INTERNAL MEDICINE SPECIALISTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>J-R16</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E58" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>Western Wayne Physicians - Livonia · PROVIDENCE PARK LIVONIA FAMILY MEDICINE</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>J-R17</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>Trinity Health IHA Medical Group Primary Care - Canton</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="3" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>J-R18</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E60" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>Trinity Health IHA Medical Group, Primary Care - Southeast Livonia</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>J-R01</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E61" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F61" s="4" t="inlineStr">
-        <is>
-          <t>BN Nandish MD</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>J-R04</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>OAK STREET HEALTH CHERRY HILL · APOLLO HEALTH SERVICES, PC · Plymouth physical therapy services</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>J-R05</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E63" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F63" s="4" t="inlineStr">
-        <is>
-          <t>Eastpointe Family Physicians · QuickDoc Urgent Care</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>J-R07</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>NORLIVO INTERNAL MEDICINE</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>J-R10</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F65" s="4" t="inlineStr">
-        <is>
-          <t>Dedicated senior Medical Center Detroit North · The family Doc</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>J-R11</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E66" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F66" s="4" t="inlineStr">
-        <is>
-          <t>Premier Medicine Medical Center - Livonia</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>J-R13</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E67" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F67" s="4" t="inlineStr">
-        <is>
-          <t>A1 Family Medicine</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>J-R14</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E68" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F68" s="4" t="inlineStr">
-        <is>
-          <t>Karma Internists · Park Family Practice - Novi · Corewell Urgent Care - Novi</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>J-R17</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F69" s="4" t="inlineStr">
-        <is>
-          <t>IHA, Primary Care - Cherry Hill Village</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>J-R18</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E70" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>CENTER FOR INTERNAL MEDICINE CONTINUITY CLINIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>J-R19</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F71" s="4" t="inlineStr">
-        <is>
-          <t>BEAUMONT FAMILY MEDICINE BELLEVILLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-21</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>J-R21</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>Producer sweep</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F72" s="4" t="inlineStr">
-        <is>
-          <t>COREWELL HEALTH  INTERNAL MEDICINE DEARBORN</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="B73" s="3" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
       </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>J-R01</t>
-        </is>
-      </c>
-      <c r="D73" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E73" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>Corwell health orthopedics Canton · CANTON FAMILY HEALTH LLC · Comprehensive Healthcare Associates and Prevention Medicine</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>J-R02</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F74" s="4" t="inlineStr">
-        <is>
-          <t>Village Medical - Novi · WEST OAKLAND INTERNISTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>J-R03</t>
-        </is>
-      </c>
-      <c r="D75" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F75" s="4" t="inlineStr">
-        <is>
-          <t>Corewell Health Wayne Hospital Internal Medicine - Canton · CANTON FOOT &amp; Ankle SPECIALISTS</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>J-R06</t>
-        </is>
-      </c>
-      <c r="D76" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F76" s="4" t="inlineStr">
-        <is>
-          <t>MEDICAL GROUP PRACTICE, PC (Olympia health)</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>J-R08</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F77" s="4" t="inlineStr">
-        <is>
-          <t>Tri County Neurology · Dedicated Senior Medical Center - Warren</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B78" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C78" s="3" t="inlineStr">
-        <is>
-          <t>J-R09</t>
-        </is>
-      </c>
-      <c r="D78" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E78" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F78" s="4" t="inlineStr">
-        <is>
-          <t>DEARBORN FAMILY CLINIC, PC · PelHam Primary Care</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B79" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C79" s="3" t="inlineStr">
-        <is>
-          <t>J-R10</t>
-        </is>
-      </c>
-      <c r="D79" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E79" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F79" s="4" t="inlineStr">
-        <is>
-          <t>Frank Lanzilote DO-Family Practice</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr">
-        <is>
-          <t>J-R12</t>
-        </is>
-      </c>
-      <c r="D80" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E80" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F80" s="4" t="inlineStr">
-        <is>
-          <t>Grand River Medical Associates</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B81" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C81" s="3" t="inlineStr">
-        <is>
-          <t>J-R15</t>
-        </is>
-      </c>
-      <c r="D81" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E81" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
-        <is>
-          <t>Roberts Orthopedic Services · SOUTHFIELD URGENT CARE · DEDICATED SENIOR MEDICAL CENTER - Southfield</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B82" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C82" s="3" t="inlineStr">
-        <is>
-          <t>J-R16</t>
-        </is>
-      </c>
-      <c r="D82" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E82" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F82" s="4" t="inlineStr">
-        <is>
-          <t>Lakes Urgent Care - Livonia</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="3" t="inlineStr">
-        <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="B83" s="3" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="C83" s="3" t="inlineStr">
-        <is>
-          <t>J-R20</t>
-        </is>
-      </c>
-      <c r="D83" s="3" t="inlineStr">
-        <is>
-          <t>Cadence revisit</t>
-        </is>
-      </c>
-      <c r="E83" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F83" s="4" t="inlineStr">
-        <is>
-          <t>TENNY INTERNAL MEDICINE, PLLC</t>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t>Open slot ×2</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr"/>
+      <c r="F44" s="9" t="inlineStr">
+        <is>
+          <t>Flex: backlog pull-forward · huddle promotes · ortho field day</t>
         </is>
       </c>
     </row>
@@ -23526,416 +22363,416 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>c19d8067-80c5-4305-b690-7e5ee2391049</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Henry Ford Athletic Medicine - Novi (relevance?)</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>Novi</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr"/>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr"/>
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>bb1e72ee-479c-42da-96ea-e71d67a1c702</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Fox Run, PC(delete)</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
         <is>
           <t>Pain</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>Novi</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr"/>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr"/>
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>c7640a25-ed3b-4097-bda5-cd89202f64a1</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Michigan Spine &amp; Brain Surgeons</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>Southfield</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>ortho opportunity</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>02dc2839-7a87-4f51-9ae8-528110ed4a8f</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>MICHIGAN SPORTS AND SPINE CENTER, PC (not of value)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Livonia</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">Competition </t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>eaa06235-6a42-4ef9-9f14-9fd1b4ed4610</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Michigan Spine &amp; Brain - Novi</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Novi</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">This would be for Ortho referrals </t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>69716ccc-b2b9-4d7b-8f77-69ecd79273be</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>PAIN MANAGEMENT ASSOCIATES OF MICHIGAN</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>Dearborn</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr"/>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr"/>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>c8be9bcd-087a-4081-93c4-84fb80a7d1d1</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Concentra Urgent Care- Novi</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>Urgent Care</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Novi</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="11" t="inlineStr">
         <is>
           <t>has own team and specific guidelines of who they can and can't sent to.</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>ec7d6518-5eb7-4fca-a6b1-325f004d1ea6</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>WATCH US GROW PEDIATRICS</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>Trenton</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr"/>
-      <c r="G10" s="9" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr"/>
+      <c r="G10" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>4e0ac17e-b678-4984-b1ba-e7825a2ed78e</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>MORSI PEDIATRICS</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>Riverview</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr"/>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="F11" s="11" t="inlineStr"/>
+      <c r="G11" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>e35d1817-e4ef-431a-a979-74b7c8e2c0f0</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>WOODHAVEN PEDIATRICS</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>Woodhaven</t>
         </is>
       </c>
-      <c r="F12" s="9" t="inlineStr"/>
-      <c r="G12" s="9" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr"/>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>fea6a17c-c68b-43db-acd7-34a4abfe0024</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Trinity Health IHA Brain &amp; Spine Surgery - Ann Arbor Campus</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>Ypsilanti</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>Ortho opportunity</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>24d003db-fb8e-4e51-adb0-77b396eef5de</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>CHILD AND ADOLESCENT CENTER, PC</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Prospect</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Prospect</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Orthopedic</t>
         </is>
       </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>Southgate</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr"/>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="F14" s="11" t="inlineStr"/>
+      <c r="G14" s="11" t="inlineStr">
         <is>
           <t>Tagged “Non-Spine” group via MMC import — out of spine rotation</t>
         </is>

</xml_diff>